<commit_message>
Rebuild the reel plan from photos of the actual room
The room is not a corner desk. It is a desk between two single beds with a
window at the far end, and the only floor space is the walkway behind the
chair. Three tripod marks move into that walkway; the two side-on marks now
stand on the right-hand bed, since there is no floor beside the chair.

Consolidate all eleven camera clips into one night session. In daylight both
beds sit in every wide shot and the reel reads as a bedroom; in darkness they
disappear and only a person lit by a screen remains, which is also the better
frame. The lamp does all the beauty/hell switching.

Add a Frame Control sheet covering what to clear and what to keep, and order
the shoot so the wide room shot is captured before the room is tidied.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/reel-shot-list.xlsx
+++ b/reel-shot-list.xlsx
@@ -10,11 +10,12 @@
     <sheet name="Shot List" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Shot Detail" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Room &amp; Light" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tripod Marks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Shoot Diary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gear &amp; Setup" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Camera Settings" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Editing Walkthrough" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Frame Control" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tripod Marks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Shoot Diary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gear &amp; Setup" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Camera Settings" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Editing Walkthrough" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,18 +48,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F2430"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Courier New"/>
-      <color rgb="001F2430"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F2430"/>
       <sz val="10"/>
     </font>
     <font>
@@ -69,20 +70,20 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="001F2430"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
+      <color rgb="001F2430"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <name val="Courier New"/>
+      <color rgb="001F2430"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="10">
@@ -163,46 +164,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -214,22 +215,22 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -612,7 +613,7 @@
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
     <col width="28" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -626,7 +627,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>11 camera clips, 2 screen recordings. Camera goes BEHIND you or to your LEFT only. Audio: "Pretty Little Baby" x bass — added inside Instagram, not in your export.</t>
+          <t>11 camera clips, 2 screen recordings. Shot almost entirely at night, because darkness hides the rest of the room. Audio: "Pretty Little Baby" x bass — added inside Instagram, not in your export.</t>
         </is>
       </c>
     </row>
@@ -744,7 +745,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>S2 Day</t>
+          <t>S1 Night</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -754,7 +755,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Behind you, high</t>
+          <t>Walkway, behind, high</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
@@ -764,7 +765,7 @@
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>You walk in, sit, set the coffee down, hands go to the keyboard.</t>
+          <t>You walk in, sit, set the water bottle down, hands to the keyboard.</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
@@ -819,7 +820,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>Behind you, high</t>
+          <t>Walkway, behind, high</t>
         </is>
       </c>
       <c r="L7" s="10" t="inlineStr">
@@ -884,7 +885,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Your left, eye height</t>
+          <t>On bed R, eye height, close</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
@@ -949,7 +950,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>Your left, eye height</t>
+          <t>On bed R, eye height, close</t>
         </is>
       </c>
       <c r="L9" s="10" t="inlineStr">
@@ -1004,7 +1005,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>S2 Day</t>
+          <t>S1 Night</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1014,7 +1015,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Your left, chest height</t>
+          <t>On bed R, chest height, back</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
@@ -1079,7 +1080,7 @@
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>Your left, chest height</t>
+          <t>On bed R, chest height, back</t>
         </is>
       </c>
       <c r="L11" s="10" t="inlineStr">
@@ -1134,7 +1135,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>S2 Day</t>
+          <t>S1 Night</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1144,7 +1145,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Behind, over your shoulder</t>
+          <t>Walkway, over your shoulder</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
@@ -1199,7 +1200,7 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>S3 Screen</t>
+          <t>S2 Screen</t>
         </is>
       </c>
       <c r="J13" s="10" t="inlineStr">
@@ -1274,7 +1275,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Behind you, high</t>
+          <t>Walkway, behind, high</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
@@ -1339,7 +1340,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Behind you, high</t>
+          <t>Walkway, behind, high</t>
         </is>
       </c>
       <c r="L15" s="10" t="inlineStr">
@@ -1349,7 +1350,7 @@
       </c>
       <c r="M15" s="11" t="inlineStr">
         <is>
-          <t>Identical frame. Warm light creeping in. Same posture, more tired.</t>
+          <t>Identical frame. Warm light creeping in from behind. More tired.</t>
         </is>
       </c>
       <c r="N15" s="11" t="inlineStr">
@@ -1394,7 +1395,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>S2 Day</t>
+          <t>S1 Night</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1404,7 +1405,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Your left, eye height</t>
+          <t>On bed R, eye height, close</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
@@ -1469,17 +1470,17 @@
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Behind, far corner, high</t>
+          <t>Walkway, far end, high</t>
         </is>
       </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>WHITE</t>
         </is>
       </c>
       <c r="M17" s="11" t="inlineStr">
         <is>
-          <t>Pull way back. The whole desk, the mess, you small in the middle of it.</t>
+          <t>Pull way back. The whole room - both beds, the mess, you small in it.</t>
         </is>
       </c>
       <c r="N17" s="11" t="inlineStr">
@@ -1524,7 +1525,7 @@
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>S3 Screen</t>
+          <t>S2 Screen</t>
         </is>
       </c>
       <c r="J18" s="13" t="inlineStr">
@@ -1604,7 +1605,7 @@
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Shot from behind (A/D/E)</t>
+          <t>Shot from the walkway (A/D/E)</t>
         </is>
       </c>
       <c r="D23" s="17">
@@ -1615,7 +1616,7 @@
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Shot from your left (B/C)</t>
+          <t>Shot from bed R (B/C)</t>
         </is>
       </c>
       <c r="D24" s="17">
@@ -1626,7 +1627,7 @@
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>Night session clips</t>
+          <t>Clips in the night session</t>
         </is>
       </c>
       <c r="D25" s="17">
@@ -1637,11 +1638,11 @@
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>Day session clips</t>
+          <t>Clips needing no camera</t>
         </is>
       </c>
       <c r="D26" s="17">
-        <f>COUNTIF(I6:I18,"S2 Day")</f>
+        <f>COUNTIF(I6:I18,"S2 Screen")</f>
         <v/>
       </c>
     </row>
@@ -1660,7 +1661,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="108" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1680,11 +1681,11 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>CLIP 1  ·  Beauty  ·  GOLD lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="46" customHeight="1">
+          <t>CLIP 1  |  Beauty  |  GOLD lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1692,11 +1693,11 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Tripod BEHIND your chair, raised high (~1.8m), tilted down. Frame: your empty chair, the grey desk, the laptop, the wall in front. Leave the top third of the frame empty for text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="46" customHeight="1">
+          <t>Tripod in the WALKWAY behind your chair, legs high (~1.7m), tilted DOWN at the desk. Frame: your empty chair, the desk, the laptop, the far wall. Tilting down is what keeps the two beds out of shot — check the edges of the frame before you record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1704,11 +1705,11 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Start recording with the chair EMPTY. Walk in from the left, sit down, put the coffee on the desk, roll the chair in, put both hands on the keyboard. Then hold still for 3 seconds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
+          <t>Start with the chair EMPTY. Walk in from the left, sit, put the water bottle on the desk, roll the chair in, both hands on the keyboard. Then hold still for 3 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1723,11 +1724,11 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>CLIP 2  ·  Hell  ·  WHITE lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+          <t>CLIP 2  |  Hell  |  WHITE lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1735,11 +1736,11 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>IDENTICAL to clip 1. Same mark, same height, same tilt. Nothing moves but the lamp mode.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+          <t>IDENTICAL to clip 1. Same spot in the walkway, same height, same tilt. Nothing moves except the lamp mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1747,11 +1748,11 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Already seated. Slumped low in the chair, one hand up on your forehead or through your hair. Screen still blank. Do nothing for 4 seconds. Stillness is the shot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
+          <t>Already seated. Slumped low, one hand up on your forehead or through your hair. Screen still blank. Do nothing for 4 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1759,18 +1760,18 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Do not act tired. Just be still and let the white light do it.</t>
+          <t>Do not act tired. Be still and let the white light do the work.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>CLIP 3  ·  Beauty  ·  Lamp OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="46" customHeight="1">
+          <t>CLIP 3  |  Beauty  |  Lamp OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1778,11 +1779,11 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Tripod to your LEFT, at eye height (~1.5m), close (about an arm's length). Frame: your face in profile, the laptop edge, the wall behind you. Screen must be the only light.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="46" customHeight="1">
+          <t>Tripod standing ON BED R (the right-hand bed), at eye height, close — about an arm's length from your face. Frame: your face in profile, edge of the laptop. Room fully dark so the background disappears entirely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1790,11 +1791,11 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Fill your terminal with green output first so it lights your face. Look at the screen, let a small real smile arrive. Do not perform it — just read the green and react.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="46" customHeight="1">
+          <t>Fill your terminal with green output first so it lights your face. Look at the screen and let a small, real smile arrive. Do not perform it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1802,18 +1803,18 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Run: python3 -m pytest tests/ -q  — the green pass block is your light source.</t>
+          <t>Run: python3 -m pytest tests/ -q — the green pass block is your only light source.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>CLIP 4  ·  Hell  ·  Lamp OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="46" customHeight="1">
+          <t>CLIP 4  |  Hell  |  Lamp OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1821,11 +1822,11 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>EXACTLY where clip 3 was. Do not touch the tripod between these two. Only the screen colour changes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="46" customHeight="1">
+          <t>EXACTLY where clip 3 was. Do not move the tripod between these two. Only the screen colour changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
       <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1837,7 +1838,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="46" customHeight="1">
+    <row r="22" ht="52" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1845,18 +1846,18 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>This pair is the best shot in the reel. It only works if the camera has not moved.</t>
+          <t>This is the best pair in the reel and it only works if nothing moved.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>CLIP 5  ·  Beauty  ·  GOLD lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="46" customHeight="1">
+          <t>CLIP 5  |  Beauty  |  GOLD lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1864,11 +1865,11 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Tripod to your LEFT, chest height (~1.2m), further back (1.5-2m) so your whole upper body and the desk are in frame, side on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="46" customHeight="1">
+          <t>Tripod on BED R, chest height, further back so your whole upper body and the desk are in frame, side on. Keep the lamp low and close to you so its pool of light does not reach the other bed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="52" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1876,11 +1877,11 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Type a few keys, hit Enter with a bit of weight, then lean back and put both arms behind your head. Hold the lean for 3 seconds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="46" customHeight="1">
+          <t>Type a few keys, hit Enter with some weight, then lean back with both arms behind your head. Hold the lean for 3 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1888,18 +1889,18 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>The lean-back is the whole shot. Hold it longer than feels natural.</t>
+          <t>The lean-back is the shot. Hold it longer than feels natural.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="18" t="inlineStr">
         <is>
-          <t>CLIP 6  ·  Hell  ·  WHITE lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="46" customHeight="1">
+          <t>CLIP 6  |  Hell  |  WHITE lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="52" customHeight="1">
       <c r="A30" s="20" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1907,11 +1908,11 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Same mark as clip 5. Same height, same distance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="46" customHeight="1">
+          <t>Same spot on BED R as clip 5. Same height, same distance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="52" customHeight="1">
       <c r="A31" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1919,11 +1920,11 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Start leaning back exactly as you ended clip 5. Then snap forward toward the laptop as though something just went wrong. Fast, one movement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="46" customHeight="1">
+          <t>Start leaning back exactly as you ended clip 5, then snap forward toward the laptop as though something has gone wrong. One fast movement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="52" customHeight="1">
       <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1938,11 +1939,11 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>CLIP 7  ·  Beauty  ·  GOLD lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="46" customHeight="1">
+          <t>CLIP 7  |  Beauty  |  GOLD lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="52" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1950,11 +1951,11 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Tripod BEHIND you, closer than Mark A, raised just above your shoulder (~1.6m), angled down at the screen. Frame: your shoulder and head bottom-left, screen filling the rest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="46" customHeight="1">
+          <t>Tripod in the WALKWAY, closer than Mark A, raised just above your shoulder (~1.6m), angled down at the screen. Frame: your shoulder and head bottom-left, screen filling the rest. This framing naturally excludes both beds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1">
       <c r="A36" s="19" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -1966,7 +1967,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="46" customHeight="1">
+    <row r="37" ht="52" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -1974,18 +1975,18 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>The screen does not need to be readable. The gesture carries it. Angle the tripod slightly off-square to the screen to avoid banding.</t>
+          <t>The screen does not need to be readable — the gesture carries it. Angle slightly off-square to the screen to avoid banding.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>CLIP 8  ·  Hell  ·  No camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="46" customHeight="1">
+          <t>CLIP 8  |  Hell  |  No camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="52" customHeight="1">
       <c r="A40" s="20" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -1993,11 +1994,11 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>Screen recording. Laptop only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="46" customHeight="1">
+          <t>Screen recording only. No tripod, no room, no setup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="52" customHeight="1">
       <c r="A41" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -2005,11 +2006,11 @@
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>Run: git blame on a file, and frame it so YOUR NAME and an old date are clearly readable. Record 8 seconds, barely moving the cursor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="46" customHeight="1">
+          <t>Run git blame on a file and frame it so YOUR NAME and an old date are clearly readable. Record 8 seconds, barely moving the cursor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="52" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -2024,11 +2025,11 @@
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>CLIP 9  ·  Beauty  ·  Lamp OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="46" customHeight="1">
+          <t>CLIP 9  |  Beauty  |  Lamp OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="52" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -2036,11 +2037,11 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Back to Mark A — behind you, high, tilted down. Identical to clips 1 and 2. Room fully dark, screen is the only light.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="46" customHeight="1">
+          <t>Back to Mark A in the walkway — behind, high, tilted down. Identical to clips 1 and 2. Room completely dark; the screen is the only light in the entire frame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="52" customHeight="1">
       <c r="A46" s="19" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -2048,11 +2049,11 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Headphones on. Sit up, hands on the keyboard, type steadily. You will read as a silhouette against the screen. Type for 8 seconds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="46" customHeight="1">
+          <t>Headphones on, sit up, hands on the keyboard, type steadily. You will read as a silhouette against the screen. Type for 8 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="52" customHeight="1">
       <c r="A47" s="19" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -2060,18 +2061,18 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Silhouettes hide everything — this is the easiest good-looking shot in the whole reel.</t>
+          <t>Total darkness erases the beds completely. This is the easiest good-looking shot you have.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>CLIP 10  ·  Hell  ·  WARM lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="46" customHeight="1">
+          <t>CLIP 10  |  Hell  |  WARM lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="52" customHeight="1">
       <c r="A50" s="20" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -2079,11 +2080,11 @@
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Mark A again, untouched. This is the same frame as clip 9.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="46" customHeight="1">
+          <t>Mark A, untouched. Same frame as clip 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="52" customHeight="1">
       <c r="A51" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -2091,11 +2092,11 @@
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>Same headphones, same seat. Switch the lamp to WARM and put it LOW and behind, so it creeps in like early light. Slump slightly. Same posture, more tired. Hold 5 seconds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="46" customHeight="1">
+          <t>Same headphones, same seat. Put the lamp on WARM and place it LOW and BEHIND you, near the window end of the walkway, so it creeps in like early light. Slump slightly. Hold 5 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="52" customHeight="1">
       <c r="A52" s="20" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -2103,18 +2104,18 @@
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>Shoot this straight after clip 9 without moving anything. The lamp change does the time-passing, so you do not need an actual sunrise.</t>
+          <t>Shoot straight after clip 9 without moving the tripod. The lamp change does the time-passing, so you never need an actual sunrise.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>CLIP 11  ·  Beauty  ·  GOLD lamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="46" customHeight="1">
+          <t>CLIP 11  |  Beauty  |  GOLD lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="52" customHeight="1">
       <c r="A55" s="19" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -2122,11 +2123,11 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Mark B again — your left, eye height, close. Same as clips 3 and 4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="46" customHeight="1">
+          <t>Mark B again — on BED R, eye height, close. Same as clips 3 and 4. Keep the gold lamp low and close to your face so the background stays dark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="52" customHeight="1">
       <c r="A56" s="19" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -2138,7 +2139,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="46" customHeight="1">
+    <row r="57" ht="52" customHeight="1">
       <c r="A57" s="19" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -2146,18 +2147,18 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Do this one first, before you have watched the demo ten times. The first reaction is the only honest one you get.</t>
+          <t>Shoot this one FIRST in the session, before you have watched the demo ten times. The first reaction is the only honest one you get.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>CLIP 12  ·  Hell  ·  Lamp OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="46" customHeight="1">
+          <t>CLIP 12  |  Hell  |  WHITE lamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="52" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -2165,11 +2166,11 @@
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>Tripod as far back into the room as it goes, raised high (~1.8m), angled down. Frame: the whole desk, the drawers, the mess, and you small in the middle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="46" customHeight="1">
+          <t>Tripod at the FAR END of the walkway, near the window, raised high (~1.8m), angled down into the room. Frame: both beds, the desk, the whole room, you small in the middle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="52" customHeight="1">
       <c r="A61" s="20" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -2181,7 +2182,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="46" customHeight="1">
+    <row r="62" ht="52" customHeight="1">
       <c r="A62" s="20" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -2189,18 +2190,18 @@
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>DO NOT TIDY THE DESK. Cups, cables and clutter are the point of this shot.</t>
+          <t>This is the ONLY shot where the whole room is meant to be visible. Shoot it FIRST, before you tidy anything — see the Frame Control sheet.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>CLIP 13  ·  Closer  ·  No camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="46" customHeight="1">
+          <t>CLIP 13  |  Closer  |  No camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="52" customHeight="1">
       <c r="A65" s="21" t="inlineStr">
         <is>
           <t>Set up</t>
@@ -2212,7 +2213,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="46" customHeight="1">
+    <row r="66" ht="52" customHeight="1">
       <c r="A66" s="21" t="inlineStr">
         <is>
           <t>Do this</t>
@@ -2220,11 +2221,11 @@
       </c>
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Run: python3 demo_guardian.py — record the whole run, then hold on the red PATCH REFUSED banner for 4 full seconds before you stop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="46" customHeight="1">
+          <t>Run python3 demo_guardian.py — record the whole run, then hold on the red PATCH REFUSED banner for 4 full seconds before stopping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="52" customHeight="1">
       <c r="A67" s="21" t="inlineStr">
         <is>
           <t>Watch out</t>
@@ -2262,13 +2263,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2281,7 +2282,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Desk against a wall, second wall on your right. That leaves only BEHIND you and your LEFT. Every shot in this reel is built from those two sides.</t>
+          <t>Desk against the far wall with a BED ON EACH SIDE. The only floor space is the walkway behind your chair. Window and balcony at the far end, behind you.</t>
         </is>
       </c>
     </row>
@@ -2295,392 +2296,441 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>                                                    </t>
+          <t xml:space="preserve">     # # # # # #  FAR WALL  # # # # # # #</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">        # # # #  WALL IN FRONT  # # # #        #</t>
+          <t xml:space="preserve">     #                                  #</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                               #</t>
+          <t xml:space="preserve">     #        [ laptop ]  [ 2nd ]       #</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">              [ laptop ]                       #  W</t>
+          <t xml:space="preserve">     #     __________________________   #</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ______________________                 #  A</t>
+          <t xml:space="preserve">     #    |      grey top            |  #</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">       |   grey desk          |                #  L</t>
+          <t xml:space="preserve">     #    |    BLUE DRAWER UNIT      |  #</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">       |______________________|                #  L</t>
+          <t xml:space="preserve">     #    |__________________________|  #</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">          [blue drawers]                       #</t>
+          <t xml:space="preserve">     #                                  #</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                               #  R</t>
+          <t xml:space="preserve">     #   _______   (chair)   _______    #</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">                (YOU)                          #  I</t>
+          <t xml:space="preserve">     #  |       |    YOU     |      |   #</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                               #  G</t>
+          <t xml:space="preserve">     #  | BED L |            | BED R|   #</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">     &lt;-- LEFT                                  #  H</t>
+          <t xml:space="preserve">     #  |       |            |  ^   |   #</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Marks B, C                               #  T</t>
+          <t xml:space="preserve">     #  |_______|     |      |__B/C_|   #</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                               #</t>
+          <t xml:space="preserve">     #             WALKWAY             #</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 ^  BEHIND -- Marks A, D, E</t>
+          <t xml:space="preserve">     #             Marks A, D          #</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>                                                    </t>
+          <t xml:space="preserve">     #                |                #</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     #             Mark E (far end)    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     #                                 #</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Side</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Open?</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     #  ~~~~~ WINDOW / BALCONY ~~~~~   #</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     # # # # # # # # # # # # # # # # # #</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Usable?</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Marks</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>What it gives you</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="44" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
-        <is>
-          <t>Behind you</t>
-        </is>
-      </c>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Walkway behind you</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="inlineStr">
+        <is>
+          <t>YES - main</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>A, D, E</t>
+        </is>
+      </c>
+      <c r="D27" s="25" t="inlineStr">
+        <is>
+          <t>Your only real floor space. Tripod goes here for 6 of the 11 camera clips. Tilt DOWN to keep both beds out of frame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>Standing on BED R</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="C24" s="25" t="inlineStr">
-        <is>
-          <t>A, D, E</t>
-        </is>
-      </c>
-      <c r="D24" s="25" t="inlineStr">
-        <is>
-          <t>Your back and shoulders, the desk, the laptop screen glowing. The classic developer frame — and the strongest look you have.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="44" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>Your left</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>B, C</t>
+        </is>
+      </c>
+      <c r="D28" s="25" t="inlineStr">
+        <is>
+          <t>There is no floor to your sides, so the bed is your tripod platform. It is stable enough for a static shot. Check the legs are not sinking before you roll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>In front of you</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>The desk is against the wall. There is nowhere to stand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>Far end of walkway</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="C25" s="25" t="inlineStr">
-        <is>
-          <t>B, C</t>
-        </is>
-      </c>
-      <c r="D25" s="25" t="inlineStr">
-        <is>
-          <t>Profile of your face lit by the screen, and your body movement in side view.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="44" customHeight="1">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
-          <t>In front</t>
-        </is>
-      </c>
-      <c r="B26" s="25" t="inlineStr">
-        <is>
-          <t>NO - wall</t>
-        </is>
-      </c>
-      <c r="C26" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="25" t="inlineStr">
-        <is>
-          <t>No room for a camera. Every straight-on shot is out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Your right</t>
-        </is>
-      </c>
-      <c r="B27" s="25" t="inlineStr">
-        <is>
-          <t>NO - wall</t>
-        </is>
-      </c>
-      <c r="C27" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D27" s="25" t="inlineStr">
-        <is>
-          <t>Blocked. Do not plan anything from this side.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="22" t="inlineStr">
-        <is>
-          <t>Your lamp is the whole beauty/hell switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="26" t="inlineStr">
-        <is>
-          <t>A 3-mode lamp is better for this than daylight, because it is repeatable. Same lamp, same position, different mode — which is literally the idea of the reel. You are not dependent on weather or a window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="inlineStr">
+        <is>
+          <t>Near the window. The only spot far enough back for the very wide shot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>Shoot at night — this is the single biggest decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>You share this room and there are two beds either side of you. In daylight they are in every wide shot and the reel reads as a bedroom. In darkness they vanish completely and all the viewer sees is a person lit by a screen. That is also the better-looking version. So every camera clip is now in ONE night session, and the lamp does all the beauty/hell switching.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>Your lamp is the beauty/hell switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Lamp mode</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Use for</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Where to put it</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Why</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="44" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="B34" s="25" t="inlineStr">
-        <is>
-          <t>All Beauty clips</t>
-        </is>
-      </c>
-      <c r="C34" s="25" t="inlineStr">
-        <is>
-          <t>Your LEFT, slightly behind, aimed at your face/desk</t>
-        </is>
-      </c>
-      <c r="D34" s="25" t="inlineStr">
-        <is>
-          <t>Warm light reads as comfort and morning. Counteracts the cold blue drawers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="44" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>WARM</t>
-        </is>
-      </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>Clip 10 only (the 'still here' shot)</t>
-        </is>
-      </c>
-      <c r="C35" s="25" t="inlineStr">
-        <is>
-          <t>Same place, dimmer if it dims</t>
-        </is>
-      </c>
-      <c r="D35" s="25" t="inlineStr">
-        <is>
-          <t>Stands in for dawn if you have no window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="44" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>WHITE</t>
-        </is>
-      </c>
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>All Hell clips</t>
-        </is>
-      </c>
-      <c r="C36" s="25" t="inlineStr">
-        <is>
-          <t>Same place, or off entirely</t>
-        </is>
-      </c>
-      <c r="D36" s="25" t="inlineStr">
-        <is>
-          <t>Cold and clinical. Reads as fluorescent, late, and unforgiving.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="44" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="B37" s="25" t="inlineStr">
+        <is>
+          <t>Beauty clips 1, 5, 7, 11</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="inlineStr">
+        <is>
+          <t>Close to you, low, on your left. Keep its pool of light off the other bed.</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Warm reads as comfort. Also fights the cold blue of the drawers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="B38" s="25" t="inlineStr">
+        <is>
+          <t>Hell clips 2, 6, 12</t>
+        </is>
+      </c>
+      <c r="C38" s="25" t="inlineStr">
+        <is>
+          <t>Same place, or higher for clip 12</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>Cold and clinical. Reads as fluorescent, late, unforgiving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>WARM</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="inlineStr">
+        <is>
+          <t>Clip 10 only</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="inlineStr">
+        <is>
+          <t>LOW and BEHIND you, near the window end</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>Creeps in like first light. Replaces needing an actual sunrise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="B37" s="25" t="inlineStr">
-        <is>
-          <t>Clips 9 and 12</t>
-        </is>
-      </c>
-      <c r="C37" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D37" s="25" t="inlineStr">
-        <is>
-          <t>Screen light only. Gives you the silhouette.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="22" t="inlineStr">
-        <is>
-          <t>Working with the colours you already have</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="26" t="inlineStr">
-        <is>
-          <t>- Grey desk - neutral, takes on whatever colour your lamp and screen give it. Ideal.</t>
+      <c r="B40" s="25" t="inlineStr">
+        <is>
+          <t>Clips 3, 4, 9</t>
+        </is>
+      </c>
+      <c r="C40" s="25" t="inlineStr">
+        <is>
+          <t>Off completely, room fully dark</t>
+        </is>
+      </c>
+      <c r="D40" s="25" t="inlineStr">
+        <is>
+          <t>Screen becomes the only light. Erases the whole room for free.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="26" t="inlineStr">
-        <is>
-          <t>- Blue drawers - read COLD. They help every Hell shot for free. Keep them in frame on those.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
+      <c r="A41" s="22" t="inlineStr">
+        <is>
+          <t>The window</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="52" customHeight="1">
       <c r="A42" s="26" t="inlineStr">
         <is>
-          <t>- For Beauty shots, the gold lamp warms the frame enough to fight the blue. Do not move the drawers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="26" t="inlineStr">
-        <is>
-          <t>- The front wall is your backdrop in Marks B and C. Keep it clear - no clutter, no posters.</t>
+          <t>It sits behind you at the far end of the walkway. You are not using it as a light source — at night it is just a dark rectangle, which is fine. Keep the curtains CLOSED for every clip so passing light and the building opposite do not change between takes. The one exception is clip 12, where a sliver of city light through the gap adds depth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Colours you already have</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>- Grey desk top - neutral. Takes on whatever colour the lamp and screen give it. Ideal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t>- Blue drawer unit - reads COLD. Free help on every Hell clip. Keep it in frame on those.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>- Pale sage wall - a clean, plain backdrop. This is genuinely good; do not hang anything on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t>- Do NOT wear blue - you will merge into the drawers. Mid-grey, charcoal or black is safest.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A40:D40"/>
-    <mergeCell ref="A30:D31"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A41:D41"/>
+  <mergeCells count="6">
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A47:D47"/>
     <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A46:D46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2692,288 +2742,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="74" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Five marks — set once on Monday, never move them</t>
+          <t>What to clear, what to keep</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All five are BEHIND you or to your LEFT, because the walls block the other two sides. Tape the floor and write the letter on the tape.</t>
+          <t>Do not strip the room bare. A room that looks like nobody lives in it kills the whole point of the reel. Clear what reads as untidy, keep what reads as 'someone works here'.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Mark</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Height</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Clips</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Must match exactly</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>Behind your chair</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="inlineStr">
-        <is>
-          <t>~1.8m, tilted down</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="inlineStr">
-        <is>
-          <t>2.5-3m back</t>
-        </is>
-      </c>
-      <c r="E5" s="25" t="inlineStr">
-        <is>
-          <t>1, 2, 9, 10</t>
-        </is>
-      </c>
-      <c r="F5" s="25" t="inlineStr">
-        <is>
-          <t>Four clips share this mark, including 9 and 10 which are the same frame minutes apart. This mark carries the reel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>Your left</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>~1.5m (eye height)</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>0.8-1m</t>
-        </is>
-      </c>
-      <c r="E6" s="25" t="inlineStr">
-        <is>
-          <t>3, 4, 11</t>
-        </is>
-      </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>Clips 3 and 4 differ ONLY in screen colour. Moving the tripod between them kills the best cut in the edit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>Your left, further back</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>~1.2m (chest)</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="inlineStr">
-        <is>
-          <t>1.5-2m</t>
-        </is>
-      </c>
-      <c r="E7" s="25" t="inlineStr">
-        <is>
-          <t>5, 6</t>
-        </is>
-      </c>
-      <c r="F7" s="25" t="inlineStr">
-        <is>
-          <t>Clip 6 starts in clip 5's ending pose. Same chair position both times.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>Behind, over your shoulder</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="inlineStr">
-        <is>
-          <t>~1.6m, angled down</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="inlineStr">
-        <is>
-          <t>0.6m behind</t>
-        </is>
-      </c>
-      <c r="E8" s="25" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="F8" s="25" t="inlineStr">
-        <is>
-          <t>Turn slightly off-square to the screen so it does not band.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Shoot clip 12 FIRST, before you tidy anything</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Clip 12 is the wide shot of the whole room and its entire content is the mess. If you tidy first you cannot get it back convincingly. Set up Mark E, shoot clip 12, then clean the room and shoot everything else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Clear it</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Clothes on bed L</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
         <is>
-          <t>Behind, far room corner</t>
-        </is>
-      </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>~1.8m, angled down</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="inlineStr">
-        <is>
-          <t>as far back as it goes</t>
-        </is>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F9" s="25" t="inlineStr">
-        <is>
-          <t>Get the drawers and the mess in frame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t>Monday setup — 30 minutes, no shooting</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>1. Unbox. Extend the legs fully once and check the head holds your phone's weight without drooping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>2. Fit the phone mount and check it grips VERTICALLY. Many mounts only hold landscape properly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>3. Set marks A to E in turn. Tape the floor under each leg. Write the letter on the tape.</t>
+          <t>Reads as laundry, not as work. Nothing else in the frame says 'developer'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>The plastic bag on the bed</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Catches the light and pulls the eye straight to it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>The blanket over the chair back</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Take it off for every clip except 12. It softens your silhouette in 9 and 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Anything on the desk you cannot name</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>If you would not describe it as part of your setup, it should not be there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Backpacks on both beds</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>Only matters for clip 12. Leave them for that, remove after.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>4. Photograph each framing FROM the phone. That photo is how you rebuild the mark later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="26" t="inlineStr">
-        <is>
-          <t>5. Write the exact leg-height setting for each mark into the Height column above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="26" t="inlineStr">
-        <is>
-          <t>6. Test at Mark B: fill the screen green, then red, and check your face actually lights up.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>7. Test the lamp in all three modes at Mark A so you know what gold, warm and white look like on camera.</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Keep it</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>The second closed laptop</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>Two machines reads as 'this person builds things'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Cables and the charger</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>Real setups have cables. Removing them looks staged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>The notebooks and pencil case</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>Texture, and they say the work is not only on screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>The water bottle</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>Your prop in clip 1 — you set it down as you sit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>The wall sockets behind the laptop</t>
+        </is>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>Nothing wrong with them. Do not try to hide them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>One thing worth saying</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="64" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>A shared bedroom with two beds and a drawer unit for a desk IS the story. Most developer content is filmed at a spotless desk with three monitors and a plant, and it is all faintly unbelievable. Building a self-hosted AI assistant from the middle of a room like this is a better version of the same reel — as long as it is intentional rather than accidental. That is all the tidying is for.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+  <mergeCells count="2">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A22:B22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2985,15 +2950,285 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Five marks — set once on Monday, never move them</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Three live in the walkway behind you. Two stand on bed R, because there is no floor to your sides. Tape the floor and write the letter on the tape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Where exactly</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Clips</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Must match exactly</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Walkway, directly behind your chair</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>~1.7m, tilted DOWN</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>1, 2, 9, 10</t>
+        </is>
+      </c>
+      <c r="E5" s="25" t="inlineStr">
+        <is>
+          <t>Four clips share this. Clips 9 and 10 are the same frame minutes apart — this mark carries the reel. Tilt down enough to lose both beds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Standing on BED R, close to you</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>~1.5m (eye height)</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>3, 4, 11</t>
+        </is>
+      </c>
+      <c r="E6" s="25" t="inlineStr">
+        <is>
+          <t>Clips 3 and 4 differ ONLY in screen colour. Moving between them kills the best cut in the edit. Mark where the legs sit on the mattress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>On BED R, further back</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>~1.2m (chest)</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>5, 6</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>Clip 6 starts in clip 5's ending pose. Same chair position both times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Walkway, close, over your shoulder</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>~1.6m, angled down</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E8" s="25" t="inlineStr">
+        <is>
+          <t>Turn slightly off-square to the screen so it does not band.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Walkway, far end near the window</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>~1.8m, angled down</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="inlineStr">
+        <is>
+          <t>The only shot where both beds SHOULD be in frame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Monday setup — 30 minutes, no shooting</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>1. Unbox. Extend the legs fully once and check the head holds your phone without drooping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>2. Check the mount grips the phone VERTICALLY. Many only hold landscape properly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>3. Set marks A, D and E in the walkway. Tape the floor under each leg, letter written on the tape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>4. For B and C, stand the tripod on bed R and mark the mattress positions with something you can find again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>5. Photograph each framing FROM the phone. That photo is how you rebuild the mark later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>6. At Mark A, tilt down until both beds are out of frame. Note that tilt angle — it is the whole trick.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>7. Test the lamp in gold, warm and white at Mark A so you know what each looks like on camera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>8. Test at Mark B: fill the screen green, then red, and check your face actually lights up.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3006,7 +3241,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Because the lamp does the lighting instead of the sun, you are no longer tied to dawn. Everything can be shot after dark except the four GOLD clips.</t>
+          <t>Because darkness hides the room and the lamp does the lighting, all 11 camera clips now fit in a single night session.</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3277,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="40" customHeight="1">
       <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Mon</t>
@@ -3074,7 +3309,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Tue</t>
@@ -3087,71 +3322,71 @@
       </c>
       <c r="C6" s="25" t="inlineStr">
         <is>
-          <t>S1 — Night session</t>
+          <t>Shoot clip 12, THEN tidy</t>
         </is>
       </c>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>60 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="E6" s="25" t="inlineStr">
         <is>
-          <t>2, 3, 4, 6, 9, 10, 12</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F6" s="25" t="inlineStr">
         <is>
-          <t>Seven clips. Room dark. Shoot 9 and 10 back to back without moving anything.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
+          <t>The wide room shot must happen before you clean. See Frame Control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>18 Aug</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>S1 — Night session (all camera)</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>75 min</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>11, 3, 4, 1, 2, 5, 6, 7, 9, 10</t>
+        </is>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Clip 11 FIRST for a genuine reaction. Then 9 and 10 back to back, lamp change only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>19 Aug</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>S2 — Day session</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="inlineStr">
-        <is>
-          <t>40 min</t>
-        </is>
-      </c>
-      <c r="E7" s="25" t="inlineStr">
-        <is>
-          <t>1, 5, 7, 11</t>
-        </is>
-      </c>
-      <c r="F7" s="25" t="inlineStr">
-        <is>
-          <t>The four GOLD clips. Lamp on gold, room otherwise normal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>19 Aug</t>
-        </is>
-      </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>S3 — Screen recordings</t>
+          <t>S2 — Screen recordings</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
@@ -3166,11 +3401,11 @@
       </c>
       <c r="F8" s="25" t="inlineStr">
         <is>
-          <t>Sitting down, no camera, no setup.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
+          <t>Sitting down, no camera, no setup. Spare day if Tuesday overran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Thu</t>
@@ -3202,7 +3437,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Fri</t>
@@ -3237,28 +3472,81 @@
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
         <is>
-          <t>If the tripod is late</t>
+          <t>Shooting order inside the night session</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>Shoot clips 8 and 13 anyway — they need no camera at all. Then slide each camera session one day later and post Saturday. Do not shoot the paired clips handheld: 1/2, 3/4, 5/6 and 9/10 only work if the frame is identical, and hands cannot do that.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
-    <row r="15"/>
+          <t>- 11 first — your genuine first reaction to the demo is only available once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>- Then 3 and 4 — same mark on bed R, only the screen colour changes. Do not move between them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>- Then 5 and 6 — move the tripod back on bed R. Clip 6 starts where clip 5 ended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>- Then 1, 2 — into the walkway at Mark A. Lamp gold, then white.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>- Then 9, 10 — same Mark A, lamp off then warm. Back to back, nothing moves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>- Then 7 — Mark D, over your shoulder. Quickest one, good to finish on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>If the tripod is late</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Shoot clips 8 and 13 anyway — they need no camera at all. Then slide the night session to Wednesday and post Saturday. Do not shoot the pairs handheld: 1/2, 3/4, 5/6 and 9/10 only work if the frame is identical, and hands cannot do that.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A13:F15"/>
+  <mergeCells count="7">
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3283,7 +3571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Short list, because the tripod and the lamp cover most of it.</t>
+          <t>Short list — the tripod and the lamp cover almost everything.</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3659,7 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Gold = Beauty. White = Hell. Warm = clip 10. Off = silhouettes.</t>
+          <t>Gold = Beauty. White = Hell. Warm = clip 10. Off = clips 3, 4, 9.</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3677,7 @@
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>Five marks, A-E, letter written on the tape.</t>
+          <t>Marks A, D, E on the floor. B and C on bed R.</t>
         </is>
       </c>
     </row>
@@ -3411,14 +3699,14 @@
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>Over-ear reads better in silhouette than buds.</t>
+          <t>Over-ear reads far better in silhouette than buds.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>Coffee cup</t>
+          <t>Water bottle</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
@@ -3428,12 +3716,12 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Clips 1, 12</t>
+          <t>Clip 1</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>Prop in clip 1, part of the mess in clip 12.</t>
+          <t>Your prop — you set it down as you sit.</t>
         </is>
       </c>
     </row>
@@ -3498,35 +3786,35 @@
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
-          <t>Wardrobe — matters more than you would think</t>
+          <t>Wardrobe</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>- Wear the SAME clothes for every clip. The pairs are supposed to be the same day.</t>
+          <t>- Same clothes for every clip. The pairs are meant to be the same day.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>- Avoid pure white — it blows out against a dark room and pulls the eye off your face.</t>
+          <t>- No blue — your drawer unit is blue and you will merge into it.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>- Avoid blue, since your drawers are already blue and you will blend into them.</t>
+          <t>- No pure white — it blows out in a dark room and drags the eye off your face.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>- A mid or dark grey or black tee is the safest choice against a grey desk and a plain wall.</t>
+          <t>- Mid-grey, charcoal or black is safest against a pale wall and a grey desk.</t>
         </is>
       </c>
     </row>
@@ -3541,32 +3829,32 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Set these once at the start of every session</t>
+          <t>Set these once at the start of the session</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>These matter more on a tripod, not less — a static frame shows every wobble in exposure.</t>
+          <t>These matter more on a tripod, not less — a static frame shows every wobble.</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3891,7 @@
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>Wipe before every session</t>
+          <t>Wipe before you start</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
@@ -3623,12 +3911,12 @@
       </c>
       <c r="C6" s="25" t="inlineStr">
         <is>
-          <t>Tap and hold your subject until AE/AF LOCK shows</t>
+          <t>Tap and hold your face until AE/AF LOCK shows</t>
         </is>
       </c>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>On a static shot, a focus hunt is glaringly obvious</t>
+          <t>In a dark room the camera hunts constantly — very visible on a static shot</t>
         </is>
       </c>
     </row>
@@ -3658,17 +3946,17 @@
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Shoot 8-10s per clip</t>
+          <t>Do NOT let it go fully dark</t>
         </is>
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>Even though you only need 2s</t>
+          <t>Keep some light on your face</t>
         </is>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>No slack to cut on the beat and no choice of take</t>
+          <t>Phone cameras get very noisy in low light. Screen light is enough; total black is not</t>
         </is>
       </c>
     </row>
@@ -3678,17 +3966,17 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Three takes of everything</t>
+          <t>Shoot 8-10s per clip</t>
         </is>
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Same setup, just roll again</t>
+          <t>Even though you only need 2s</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>The third take is always the natural one</t>
+          <t>No slack to cut on the beat and no choice of take</t>
         </is>
       </c>
     </row>
@@ -3698,17 +3986,17 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>Never digital zoom</t>
+          <t>Three takes of everything</t>
         </is>
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Move the tripod instead</t>
+          <t>Same setup, just roll again</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>Zoom is cropping — soft, mushy footage</t>
+          <t>The third take is always the natural one</t>
         </is>
       </c>
     </row>
@@ -3718,17 +4006,17 @@
       </c>
       <c r="B11" s="24" t="inlineStr">
         <is>
-          <t>Shoot vertical natively</t>
+          <t>Never digital zoom</t>
         </is>
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>9:16 from the start</t>
+          <t>Move the tripod instead</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>Cropping landscape throws away most of your resolution</t>
+          <t>Zoom is cropping — soft, mushy footage</t>
         </is>
       </c>
     </row>
@@ -3738,17 +4026,17 @@
       </c>
       <c r="B12" s="24" t="inlineStr">
         <is>
-          <t>Do Not Disturb on</t>
+          <t>Shoot vertical natively</t>
         </is>
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Before every take</t>
+          <t>9:16 from the start</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>One notification banner and you reshoot</t>
+          <t>Cropping landscape throws away most of your resolution</t>
         </is>
       </c>
     </row>
@@ -3758,17 +4046,17 @@
       </c>
       <c r="B13" s="24" t="inlineStr">
         <is>
-          <t>Lock screen brightness</t>
+          <t>Do Not Disturb on</t>
         </is>
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>Turn off auto-brightness on the laptop</t>
+          <t>Before every take</t>
         </is>
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
-          <t>Your key light changes mid-shot — fatal for clips 3, 4, 9</t>
+          <t>One notification banner and you reshoot</t>
         </is>
       </c>
     </row>
@@ -3778,17 +4066,37 @@
       </c>
       <c r="B14" s="24" t="inlineStr">
         <is>
-          <t>Photograph every framing</t>
+          <t>Lock laptop brightness</t>
         </is>
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>On Monday, at all five marks</t>
+          <t>Turn off auto-brightness</t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>You cannot rebuild Mark A from memory two days later</t>
+          <t>Your key light changes mid-shot — fatal for clips 3, 4, 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Check the frame edges</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>Before every take at Mark A</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>A corner of a bed creeping in is the easiest mistake to make in this room</t>
         </is>
       </c>
     </row>
@@ -3797,7 +4105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3867,7 +4175,7 @@
       </c>
       <c r="D6" s="25" t="inlineStr">
         <is>
-          <t>Play Store / App Store, search 'VN Video Editor'. Free, and it does not put a watermark on your export. NOTE: CapCut is what most tutorials use, but it is not available in India — VN is the equivalent and works everywhere.</t>
+          <t>Play Store / App Store, search 'VN Video Editor'. Free, and no watermark on export. NOTE: CapCut is what most tutorials use, but it is not available in India — VN is the equivalent and works everywhere.</t>
         </is>
       </c>
     </row>
@@ -3883,7 +4191,7 @@
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Find the 'Pretty Little Baby' bass/sped-up remix you want and save the audio file to your device. You need it inside the editor to cut against, even though the final reel uses Instagram's copy.</t>
+          <t>Find the 'Pretty Little Baby' bass/sped-up remix you want and save the audio to your device. You need it inside the editor to cut against, even though the final reel uses Instagram's copy.</t>
         </is>
       </c>
     </row>
@@ -3899,7 +4207,7 @@
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>Play it and write down the timestamp you want to open on — for example 0:12. You will need this exact number in step 24.</t>
+          <t>Play it and write down the timestamp you want to open on — for example 0:12. You need this exact number again at step 25.</t>
         </is>
       </c>
     </row>
@@ -3922,7 +4230,7 @@
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>You will have ~40 files from 3 takes each. In your gallery, pick the one keeper per shot and put the 13 winners in an album called 'reel'.</t>
+          <t>You will have around 40 files from 3 takes each. In your gallery, pick the one keeper per shot and put the 13 winners in an album called 'reel'.</t>
         </is>
       </c>
     </row>
@@ -3938,7 +4246,7 @@
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>Fifteen minutes here saves about an hour of scrolling through a crowded timeline. This is the step beginners skip and then drown.</t>
+          <t>Fifteen minutes here saves about an hour of scrolling a crowded timeline. This is the step beginners skip and then drown.</t>
         </is>
       </c>
     </row>
@@ -3977,7 +4285,7 @@
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>Select them from the 'reel' album, in clip order 1 to 13. They land on the timeline at the bottom of the screen.</t>
+          <t>Select them from the 'reel' album in clip order 1 to 13. They land on the timeline at the bottom of the screen.</t>
         </is>
       </c>
     </row>
@@ -3993,7 +4301,7 @@
       </c>
       <c r="D15" s="25" t="inlineStr">
         <is>
-          <t>Tap Music (or Audio) then 'From device' and pick your saved track. It appears as a second bar under your video.</t>
+          <t>Tap Music (or Audio), then 'From device', and pick your saved track. It appears as a second bar under your video.</t>
         </is>
       </c>
     </row>
@@ -4048,7 +4356,7 @@
       </c>
       <c r="D19" s="25" t="inlineStr">
         <is>
-          <t>Markers first, footage second. If you place clips first and sync afterwards you will fight it the entire way through.</t>
+          <t>Markers first, footage second. Place clips first and try to sync afterwards and you will fight it the whole way through.</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4379,7 @@
       </c>
       <c r="D21" s="25" t="inlineStr">
         <is>
-          <t>Then drag its right-hand edge left until the clip ENDS on the first marker. It will snap.</t>
+          <t>Then drag its right-hand edge left until the clip ENDS on the first marker. It snaps.</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4395,7 @@
       </c>
       <c r="D22" s="25" t="inlineStr">
         <is>
-          <t>Clip 2 ends on marker 2, clip 3 on marker 3, and so on.</t>
+          <t>Clip 2 ends on marker 2, clip 3 on marker 3, and so on down the line.</t>
         </is>
       </c>
     </row>
@@ -4103,7 +4411,7 @@
       </c>
       <c r="D23" s="25" t="inlineStr">
         <is>
-          <t>Even-numbered clips (the Hell ones) should land on the heavy hits.</t>
+          <t>The even-numbered clips are the Hell ones — they should land on the heavy hits.</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4530,7 @@
       </c>
       <c r="D31" s="25" t="inlineStr">
         <is>
-          <t>No transitions, no filters, no zoom effects. Hard cuts only. Over-effecting is the single clearest sign of a first edit.</t>
+          <t>No transitions, no filters, no zoom effects. Hard cuts only. Over-effecting is the clearest sign of a first edit.</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4608,7 @@
       </c>
       <c r="D37" s="25" t="inlineStr">
         <is>
-          <t>Set it to start at the number you wrote down in step 3. This is what re-aligns your cuts to the music.</t>
+          <t>Set it to start at the number you wrote down at step 3. This is what re-aligns your cuts to the music.</t>
         </is>
       </c>
     </row>
@@ -4369,7 +4677,7 @@
     <row r="44">
       <c r="A44" s="26" t="inlineStr">
         <is>
-          <t>- The second one takes about 40 minutes. The fourth takes 20. It gets fast quickly.</t>
+          <t>- The second takes about 40 minutes. The fourth takes 20. It gets fast quickly.</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4691,7 @@
     <row r="46">
       <c r="A46" s="26" t="inlineStr">
         <is>
-          <t>- Watch the finished reel MUTED before you post. If it does not read without sound, the text is wrong.</t>
+          <t>- Watch it MUTED before you post. If it does not read without sound, the text is wrong.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Give the tripod marks measured positions and put the spare kit to work
Replace the vague mark descriptions with positions measured back from the
front edge of the desk, which is the one landmark in the room that never
moves. Add a plan-view diagram showing all five, a no-tape-measure method
for setting them, and blank columns to record the distances actually used
once the framing looks right on Monday.

Use the second laptop as the screen that lights up in clip 6 — the phone is
the camera, so the alert had to land somewhere it could film. Add the tablet
and spare headphones as desk dressing, with a note against using the tablet
as a second camera inside a paired shot.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLTsBRbD5LTCiR7DCK43kP
</commit_message>
<xml_diff>
--- a/reel-shot-list.xlsx
+++ b/reel-shot-list.xlsx
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,13 +226,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1920,7 +1927,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Start leaning back exactly as you ended clip 5, then snap forward toward the laptop as though something has gone wrong. One fast movement.</t>
+          <t>Start leaning back exactly as you ended clip 5. Then LAPTOP 2 lights up beside you with notifications, and you snap forward toward it. One fast movement.</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1939,7 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Starting in clip 5's end position is what makes the cut land.</t>
+          <t>This is what the second laptop is for. Your phone is the camera, so the thing that lights up has to be a screen you are not holding. Queue the alerts on laptop 2 before you roll.</t>
         </is>
       </c>
     </row>
@@ -2742,11 +2749,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="74" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2924,21 +2932,178 @@
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
+          <t>Dress the desk with the kit you already own</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Two laptops, a tablet with a Bluetooth keyboard and two pairs of wired headphones is genuinely a lot of kit in frame. Used deliberately it turns a bedroom desk into something that reads as a workstation, which is most of the production value you are missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Where to put it</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>What it does for the shot</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Laptop 1</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="inlineStr">
+        <is>
+          <t>Centre, in front of you — your working machine</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
+        <is>
+          <t>The hero. Every screen-lit shot uses this as the light source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Laptop 2</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="inlineStr">
+        <is>
+          <t>Open, angled, to your RIGHT</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>This is the screen that lights up in clip 6. It also solves the problem that your phone is the camera and cannot film itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>Tablet + BT keyboard</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="inlineStr">
+        <is>
+          <t>Propped upright to your LEFT, slightly behind laptop 1</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="inlineStr">
+        <is>
+          <t>Adds a third glowing rectangle and depth to the frame. Put the Guardian demo output on it so there is something red or green in the background.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>Headphones 1</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="inlineStr">
+        <is>
+          <t>Worn — clips 9 and 10</t>
+        </is>
+      </c>
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>Over-ear reads far better in silhouette than buds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Headphones 2</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="inlineStr">
+        <is>
+          <t>Hanging off the desk edge or coiled by laptop 2</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Small lived-in detail. Costs nothing, adds texture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="40" customHeight="1">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>Wired earbuds</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="inlineStr">
+        <is>
+          <t>In your hand, off camera</t>
+        </is>
+      </c>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>Volume button is your shutter remote — you are in almost every frame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>Three lit screens is the sweet spot. More than that and it reads as a stock photo of a hacker. Keep all three on the SAME brightness so no single one blows out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Can the tablet be a second camera?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="26" t="inlineStr">
+        <is>
+          <t>Only for shots that stand alone — clip 12, or a bonus angle you might not use. Never for one half of a pair. Two different cameras give you different colour and sharpness, and clips 3 and 4 are supposed to look identical apart from the screen. Mixing cameras inside a pair is the one thing that would break the reel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
           <t>One thing worth saying</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="64" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
+    <row r="37" ht="64" customHeight="1">
+      <c r="A37" s="26" t="inlineStr">
         <is>
           <t>A shared bedroom with two beds and a drawer unit for a desk IS the story. Most developer content is filmed at a spotless desk with three monitors and a plant, and it is all faintly unbelievable. Building a self-hosted AI assistant from the middle of a room like this is a better version of the same reel — as long as it is intentional rather than accidental. That is all the tidying is for.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A34:C34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2950,265 +3115,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Five marks — set once on Monday, never move them</t>
+          <t>Where exactly the tripod stands</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Three live in the walkway behind you. Two stand on bed R, because there is no floor to your sides. Tape the floor and write the letter on the tape.</t>
+          <t>Every position is measured from the FRONT EDGE OF YOUR DESK, straight back along the walkway. That edge never moves, so it is the one landmark you can always find again.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Plan view — looking down at the room</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  # # # # # # # # # #  FAR WALL  # # # # # # # # # #</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #                                                #</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #      [laptop]              [2nd laptop]        #</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #   ==========================================   #</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |              DESK  (grey top)            |  #</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |            BLUE DRAWER UNIT              |  #</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |__________________________________________|  #</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #        ^^^ FRONT EDGE OF DESK = 0.0m ^^^       #</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #                                                #</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #   _________       (chair)        _________     #</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |         |      [ YOU ]       |         |    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |         |                    |         |    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |  BED L  |     * D  0.9m      |  BED R  |    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |         |                    |  *B 0.6m|    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |         |                    |         |    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |         |     * A  1.8m      |  *C 1.5m|    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #  |_________|                    |_________|    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #                                                #</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #                 * E  3.0m                      #</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #                 (or as far back as it goes)    #</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #                                                #</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #      ~ ~ ~ ~ WINDOW / BALCONY ~ ~ ~ ~          #</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  # # # # # # # # # # # # # # # # # # # # # # # # ##</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A, D, E  stand on the WALKWAY FLOOR, centred on the laptop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  B, C     stand ON TOP OF BED R, level with / behind the chair.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Mark</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Where exactly</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Height</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Stands on</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Back from desk edge</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Side to side</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Leg height</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Tilt</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Clips</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Must match exactly</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>ACTUAL back (fill Mon)</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>ACTUAL height (fill Mon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="36" customHeight="1">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>Walkway, directly behind your chair</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="inlineStr">
-        <is>
-          <t>~1.7m, tilted DOWN</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
+        <is>
+          <t>Walkway floor</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>1.8 m</t>
+        </is>
+      </c>
+      <c r="D34" s="25" t="inlineStr">
+        <is>
+          <t>Centred on the laptop</t>
+        </is>
+      </c>
+      <c r="E34" s="28" t="inlineStr">
+        <is>
+          <t>1.7 m</t>
+        </is>
+      </c>
+      <c r="F34" s="25" t="inlineStr">
+        <is>
+          <t>Tilt DOWN ~25 deg</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="inlineStr">
         <is>
           <t>1, 2, 9, 10</t>
         </is>
       </c>
-      <c r="E5" s="25" t="inlineStr">
-        <is>
-          <t>Four clips share this. Clips 9 and 10 are the same frame minutes apart — this mark carries the reel. Tilt down enough to lose both beds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="H34" s="29" t="inlineStr"/>
+      <c r="I34" s="29" t="inlineStr"/>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="27" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>Standing on BED R, close to you</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>~1.5m (eye height)</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>On top of BED R</t>
+        </is>
+      </c>
+      <c r="C35" s="28" t="inlineStr">
+        <is>
+          <t>0.6 m</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="inlineStr">
+        <is>
+          <t>Right edge of the walkway, close in</t>
+        </is>
+      </c>
+      <c r="E35" s="28" t="inlineStr">
+        <is>
+          <t>1.5 m</t>
+        </is>
+      </c>
+      <c r="F35" s="25" t="inlineStr">
+        <is>
+          <t>Level, pointed at your face</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="inlineStr">
         <is>
           <t>3, 4, 11</t>
         </is>
       </c>
-      <c r="E6" s="25" t="inlineStr">
-        <is>
-          <t>Clips 3 and 4 differ ONLY in screen colour. Moving between them kills the best cut in the edit. Mark where the legs sit on the mattress.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="H35" s="29" t="inlineStr"/>
+      <c r="I35" s="29" t="inlineStr"/>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="27" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>On BED R, further back</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>~1.2m (chest)</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
+        <is>
+          <t>On top of BED R</t>
+        </is>
+      </c>
+      <c r="C36" s="28" t="inlineStr">
+        <is>
+          <t>1.5 m</t>
+        </is>
+      </c>
+      <c r="D36" s="25" t="inlineStr">
+        <is>
+          <t>Right edge, further out</t>
+        </is>
+      </c>
+      <c r="E36" s="28" t="inlineStr">
+        <is>
+          <t>1.2 m</t>
+        </is>
+      </c>
+      <c r="F36" s="25" t="inlineStr">
+        <is>
+          <t>Level, side on</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="inlineStr">
         <is>
           <t>5, 6</t>
         </is>
       </c>
-      <c r="E7" s="25" t="inlineStr">
-        <is>
-          <t>Clip 6 starts in clip 5's ending pose. Same chair position both times.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="H36" s="29" t="inlineStr"/>
+      <c r="I36" s="29" t="inlineStr"/>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="27" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>Walkway, close, over your shoulder</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="inlineStr">
-        <is>
-          <t>~1.6m, angled down</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
+        <is>
+          <t>Walkway floor</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="inlineStr">
+        <is>
+          <t>0.9 m</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Just right of your head</t>
+        </is>
+      </c>
+      <c r="E37" s="28" t="inlineStr">
+        <is>
+          <t>1.6 m</t>
+        </is>
+      </c>
+      <c r="F37" s="25" t="inlineStr">
+        <is>
+          <t>Tilt DOWN ~35 deg at the screen</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="E8" s="25" t="inlineStr">
-        <is>
-          <t>Turn slightly off-square to the screen so it does not band.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="H37" s="29" t="inlineStr"/>
+      <c r="I37" s="29" t="inlineStr"/>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="27" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
-        <is>
-          <t>Walkway, far end near the window</t>
-        </is>
-      </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>~1.8m, angled down</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="B38" s="25" t="inlineStr">
+        <is>
+          <t>Walkway floor</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="inlineStr">
+        <is>
+          <t>3.0 m</t>
+        </is>
+      </c>
+      <c r="D38" s="25" t="inlineStr">
+        <is>
+          <t>Centred on the walkway</t>
+        </is>
+      </c>
+      <c r="E38" s="28" t="inlineStr">
+        <is>
+          <t>1.8 m</t>
+        </is>
+      </c>
+      <c r="F38" s="25" t="inlineStr">
+        <is>
+          <t>Tilt DOWN ~20 deg</t>
+        </is>
+      </c>
+      <c r="G38" s="28" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>The only shot where both beds SHOULD be in frame.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="H38" s="29" t="inlineStr"/>
+      <c r="I38" s="29" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>The numbers above are starting points, not gospel</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t>Your room may be narrower or deeper than I have guessed from the photos. On Monday, set each mark, look at the framing, adjust until it looks right, THEN measure what you actually ended up with and write it into the two blue columns. After that you never guess again — you just read your own numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="inlineStr">
+        <is>
+          <t>How to measure without a tape measure</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="26" t="inlineStr">
+        <is>
+          <t>- One normal walking step is roughly 0.75 m. Mark A is about 2 steps back from the desk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>- A single bed is about 0.9 m wide - use the bed edge as your ruler for side-to-side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t>- For leg height, count the number of leg segments you extend and write THAT down instead of cm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>- For tilt, photograph the tripod head from the side once it looks right. Match the photo later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>Marking them physically</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
+      <c r="A50" s="26" t="inlineStr">
+        <is>
+          <t>- FLOOR (A, D, E): tape a cross where the FRONT leg sits, and write the letter on the tape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>- Two legs forward, one leg back, every time - so a single taped cross is enough to rebuild it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="26" t="inlineStr">
+        <is>
+          <t>- BED (B, C): you cannot tape a mattress usefully. Instead line the front leg up with a fixed point - the edge of the pillow, a seam in the bedsheet, the corner of the bed frame - and write down which one in the blue column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t>- Photograph every framing from the phone on Monday. That photo is your real reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>Monday setup — 30 minutes, no shooting</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+    <row r="56" ht="26" customHeight="1">
+      <c r="A56" s="26" t="inlineStr">
         <is>
           <t>1. Unbox. Extend the legs fully once and check the head holds your phone without drooping.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+    <row r="57" ht="26" customHeight="1">
+      <c r="A57" s="26" t="inlineStr">
         <is>
           <t>2. Check the mount grips the phone VERTICALLY. Many only hold landscape properly.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>3. Set marks A, D and E in the walkway. Tape the floor under each leg, letter written on the tape.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>4. For B and C, stand the tripod on bed R and mark the mattress positions with something you can find again.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="26" t="inlineStr">
-        <is>
-          <t>5. Photograph each framing FROM the phone. That photo is how you rebuild the mark later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="26" t="inlineStr">
-        <is>
-          <t>6. At Mark A, tilt down until both beds are out of frame. Note that tilt angle — it is the whole trick.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>7. Test the lamp in gold, warm and white at Mark A so you know what each looks like on camera.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="26" t="inlineStr">
-        <is>
-          <t>8. Test at Mark B: fill the screen green, then red, and check your face actually lights up.</t>
+    <row r="58" ht="26" customHeight="1">
+      <c r="A58" s="26" t="inlineStr">
+        <is>
+          <t>3. Set A, D, E on the walkway floor. Tape a cross under the front leg, letter on the tape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="26" customHeight="1">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
+          <t>4. Set B and C on bed R. Line the front leg to a fixed point and write it in the blue column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="26" customHeight="1">
+      <c r="A60" s="26" t="inlineStr">
+        <is>
+          <t>5. At Mark A, tilt down until BOTH BEDS are out of frame. This is the most important setting in the whole shoot - note the tilt and photograph the tripod head from the side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>6. Photograph each framing FROM the phone. Five reference photos, one per mark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="26" customHeight="1">
+      <c r="A62" s="26" t="inlineStr">
+        <is>
+          <t>7. Measure what you actually used and fill in the two blue columns above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>8. Test the lamp in gold, warm and white at Mark A so you know what each looks like on camera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="26" customHeight="1">
+      <c r="A64" s="26" t="inlineStr">
+        <is>
+          <t>9. Test at Mark B: fill the screen green, then red, and check your face actually lights up.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A18:E18"/>
+  <mergeCells count="18">
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="A64:I64"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A51:I51"/>
+    <mergeCell ref="A63:I63"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A60:I60"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A61:I61"/>
+    <mergeCell ref="A58:I58"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A62:I62"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3684,7 +4219,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
         <is>
-          <t>Headphones</t>
+          <t>Laptop 2</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
@@ -3694,19 +4229,19 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>Clips 9, 10</t>
+          <t>Clip 6, and desk dressing</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>Over-ear reads far better in silhouette than buds.</t>
+          <t>The screen that lights up in clip 6. Queue the alerts on it before you roll.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
-          <t>Water bottle</t>
+          <t>Tablet + BT keyboard</t>
         </is>
       </c>
       <c r="B10" s="25" t="inlineStr">
@@ -3716,19 +4251,19 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Clip 1</t>
+          <t>Desk dressing</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>Your prop — you set it down as you sit.</t>
+          <t>Propped to your left. Put the Guardian output on it for background colour.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>Your t-shirt</t>
+          <t>Headphones x2</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
@@ -3738,55 +4273,92 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>Lens cloth</t>
+          <t>Clips 9, 10 + dressing</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">
         <is>
-          <t>Biggest free quality jump there is.</t>
+          <t>Wear one, hang the other off the desk edge. Over-ear beats buds in silhouette.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="24" t="inlineStr">
         <is>
-          <t>Wired earbuds</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="inlineStr"/>
+          <t>Water bottle</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Shutter remote</t>
+          <t>Clip 1</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>Volume button fires the shutter — useful since you are in almost every frame.</t>
+          <t>Your prop — you set it down as you sit.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>VN Video Editor</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="inlineStr"/>
+          <t>Your t-shirt</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
+          <t>Lens cloth</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>Biggest free quality jump there is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Wired earbuds</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr"/>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Shutter remote</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>Volume button fires the shutter — useful since you are in almost every frame.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Wardrobe</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr"/>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
           <t>The edit</t>
         </is>
       </c>
-      <c r="D13" s="25" t="inlineStr">
+      <c r="D15" s="25" t="inlineStr">
         <is>
           <t>Free, no watermark. See Editing Walkthrough.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr">
-        <is>
-          <t>Wardrobe</t>
         </is>
       </c>
     </row>
@@ -4157,15 +4729,15 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>BEFORE YOU START</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="28" t="inlineStr"/>
-      <c r="B6" s="29" t="n">
+      <c r="A6" s="32" t="inlineStr"/>
+      <c r="B6" s="28" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="24" t="inlineStr">
@@ -4180,8 +4752,8 @@
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="28" t="inlineStr"/>
-      <c r="B7" s="29" t="n">
+      <c r="A7" s="32" t="inlineStr"/>
+      <c r="B7" s="28" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="24" t="inlineStr">
@@ -4196,8 +4768,8 @@
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="28" t="inlineStr"/>
-      <c r="B8" s="29" t="n">
+      <c r="A8" s="32" t="inlineStr"/>
+      <c r="B8" s="28" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="24" t="inlineStr">
@@ -4212,15 +4784,15 @@
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>SORT YOUR FOOTAGE</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="28" t="inlineStr"/>
-      <c r="B10" s="29" t="n">
+      <c r="A10" s="32" t="inlineStr"/>
+      <c r="B10" s="28" t="n">
         <v>4</v>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -4235,8 +4807,8 @@
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="28" t="inlineStr"/>
-      <c r="B11" s="29" t="n">
+      <c r="A11" s="32" t="inlineStr"/>
+      <c r="B11" s="28" t="n">
         <v>5</v>
       </c>
       <c r="C11" s="24" t="inlineStr">
@@ -4251,15 +4823,15 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>SET UP THE PROJECT</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="28" t="inlineStr"/>
-      <c r="B13" s="29" t="n">
+      <c r="A13" s="32" t="inlineStr"/>
+      <c r="B13" s="28" t="n">
         <v>6</v>
       </c>
       <c r="C13" s="24" t="inlineStr">
@@ -4274,8 +4846,8 @@
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="28" t="inlineStr"/>
-      <c r="B14" s="29" t="n">
+      <c r="A14" s="32" t="inlineStr"/>
+      <c r="B14" s="28" t="n">
         <v>7</v>
       </c>
       <c r="C14" s="24" t="inlineStr">
@@ -4290,8 +4862,8 @@
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="28" t="inlineStr"/>
-      <c r="B15" s="29" t="n">
+      <c r="A15" s="32" t="inlineStr"/>
+      <c r="B15" s="28" t="n">
         <v>8</v>
       </c>
       <c r="C15" s="24" t="inlineStr">
@@ -4306,15 +4878,15 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>BEAT MARKERS — the one skill that matters</t>
         </is>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="28" t="inlineStr"/>
-      <c r="B17" s="29" t="n">
+      <c r="A17" s="32" t="inlineStr"/>
+      <c r="B17" s="28" t="n">
         <v>9</v>
       </c>
       <c r="C17" s="24" t="inlineStr">
@@ -4329,8 +4901,8 @@
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="28" t="inlineStr"/>
-      <c r="B18" s="29" t="n">
+      <c r="A18" s="32" t="inlineStr"/>
+      <c r="B18" s="28" t="n">
         <v>10</v>
       </c>
       <c r="C18" s="24" t="inlineStr">
@@ -4345,8 +4917,8 @@
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="28" t="inlineStr"/>
-      <c r="B19" s="29" t="n">
+      <c r="A19" s="32" t="inlineStr"/>
+      <c r="B19" s="28" t="n">
         <v>11</v>
       </c>
       <c r="C19" s="24" t="inlineStr">
@@ -4361,15 +4933,15 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>PLACE THE CLIPS</t>
         </is>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
-      <c r="A21" s="28" t="inlineStr"/>
-      <c r="B21" s="29" t="n">
+      <c r="A21" s="32" t="inlineStr"/>
+      <c r="B21" s="28" t="n">
         <v>12</v>
       </c>
       <c r="C21" s="24" t="inlineStr">
@@ -4384,8 +4956,8 @@
       </c>
     </row>
     <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="28" t="inlineStr"/>
-      <c r="B22" s="29" t="n">
+      <c r="A22" s="32" t="inlineStr"/>
+      <c r="B22" s="28" t="n">
         <v>13</v>
       </c>
       <c r="C22" s="24" t="inlineStr">
@@ -4400,8 +4972,8 @@
       </c>
     </row>
     <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="28" t="inlineStr"/>
-      <c r="B23" s="29" t="n">
+      <c r="A23" s="32" t="inlineStr"/>
+      <c r="B23" s="28" t="n">
         <v>14</v>
       </c>
       <c r="C23" s="24" t="inlineStr">
@@ -4416,8 +4988,8 @@
       </c>
     </row>
     <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="28" t="inlineStr"/>
-      <c r="B24" s="29" t="n">
+      <c r="A24" s="32" t="inlineStr"/>
+      <c r="B24" s="28" t="n">
         <v>15</v>
       </c>
       <c r="C24" s="24" t="inlineStr">
@@ -4432,8 +5004,8 @@
       </c>
     </row>
     <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="28" t="inlineStr"/>
-      <c r="B25" s="29" t="n">
+      <c r="A25" s="32" t="inlineStr"/>
+      <c r="B25" s="28" t="n">
         <v>16</v>
       </c>
       <c r="C25" s="24" t="inlineStr">
@@ -4448,15 +5020,15 @@
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>TEXT</t>
         </is>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1">
-      <c r="A27" s="28" t="inlineStr"/>
-      <c r="B27" s="29" t="n">
+      <c r="A27" s="32" t="inlineStr"/>
+      <c r="B27" s="28" t="n">
         <v>17</v>
       </c>
       <c r="C27" s="24" t="inlineStr">
@@ -4471,8 +5043,8 @@
       </c>
     </row>
     <row r="28" ht="42" customHeight="1">
-      <c r="A28" s="28" t="inlineStr"/>
-      <c r="B28" s="29" t="n">
+      <c r="A28" s="32" t="inlineStr"/>
+      <c r="B28" s="28" t="n">
         <v>18</v>
       </c>
       <c r="C28" s="24" t="inlineStr">
@@ -4487,8 +5059,8 @@
       </c>
     </row>
     <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="28" t="inlineStr"/>
-      <c r="B29" s="29" t="n">
+      <c r="A29" s="32" t="inlineStr"/>
+      <c r="B29" s="28" t="n">
         <v>19</v>
       </c>
       <c r="C29" s="24" t="inlineStr">
@@ -4503,8 +5075,8 @@
       </c>
     </row>
     <row r="30" ht="42" customHeight="1">
-      <c r="A30" s="28" t="inlineStr"/>
-      <c r="B30" s="29" t="n">
+      <c r="A30" s="32" t="inlineStr"/>
+      <c r="B30" s="28" t="n">
         <v>20</v>
       </c>
       <c r="C30" s="24" t="inlineStr">
@@ -4519,8 +5091,8 @@
       </c>
     </row>
     <row r="31" ht="42" customHeight="1">
-      <c r="A31" s="28" t="inlineStr"/>
-      <c r="B31" s="29" t="n">
+      <c r="A31" s="32" t="inlineStr"/>
+      <c r="B31" s="28" t="n">
         <v>21</v>
       </c>
       <c r="C31" s="24" t="inlineStr">
@@ -4535,15 +5107,15 @@
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="27" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>EXPORT</t>
         </is>
       </c>
     </row>
     <row r="33" ht="42" customHeight="1">
-      <c r="A33" s="28" t="inlineStr"/>
-      <c r="B33" s="29" t="n">
+      <c r="A33" s="32" t="inlineStr"/>
+      <c r="B33" s="28" t="n">
         <v>22</v>
       </c>
       <c r="C33" s="24" t="inlineStr">
@@ -4558,8 +5130,8 @@
       </c>
     </row>
     <row r="34" ht="42" customHeight="1">
-      <c r="A34" s="28" t="inlineStr"/>
-      <c r="B34" s="29" t="n">
+      <c r="A34" s="32" t="inlineStr"/>
+      <c r="B34" s="28" t="n">
         <v>23</v>
       </c>
       <c r="C34" s="24" t="inlineStr">
@@ -4574,15 +5146,15 @@
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="27" t="inlineStr">
+      <c r="A35" s="31" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
     </row>
     <row r="36" ht="42" customHeight="1">
-      <c r="A36" s="28" t="inlineStr"/>
-      <c r="B36" s="29" t="n">
+      <c r="A36" s="32" t="inlineStr"/>
+      <c r="B36" s="28" t="n">
         <v>24</v>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -4597,8 +5169,8 @@
       </c>
     </row>
     <row r="37" ht="42" customHeight="1">
-      <c r="A37" s="28" t="inlineStr"/>
-      <c r="B37" s="29" t="n">
+      <c r="A37" s="32" t="inlineStr"/>
+      <c r="B37" s="28" t="n">
         <v>25</v>
       </c>
       <c r="C37" s="24" t="inlineStr">
@@ -4613,8 +5185,8 @@
       </c>
     </row>
     <row r="38" ht="42" customHeight="1">
-      <c r="A38" s="28" t="inlineStr"/>
-      <c r="B38" s="29" t="n">
+      <c r="A38" s="32" t="inlineStr"/>
+      <c r="B38" s="28" t="n">
         <v>26</v>
       </c>
       <c r="C38" s="24" t="inlineStr">
@@ -4629,8 +5201,8 @@
       </c>
     </row>
     <row r="39" ht="42" customHeight="1">
-      <c r="A39" s="28" t="inlineStr"/>
-      <c r="B39" s="29" t="n">
+      <c r="A39" s="32" t="inlineStr"/>
+      <c r="B39" s="28" t="n">
         <v>27</v>
       </c>
       <c r="C39" s="24" t="inlineStr">
@@ -4645,8 +5217,8 @@
       </c>
     </row>
     <row r="40" ht="42" customHeight="1">
-      <c r="A40" s="28" t="inlineStr"/>
-      <c r="B40" s="29" t="n">
+      <c r="A40" s="32" t="inlineStr"/>
+      <c r="B40" s="28" t="n">
         <v>28</v>
       </c>
       <c r="C40" s="24" t="inlineStr">

</xml_diff>